<commit_message>
data(gold): TCC refeito + rotulado + ground_truth pos-poda (36 joined, 20 disc)
Template regenerado (tipo=file_type puro) preservando rotulos; 4 off-by-one
corrigidos com confirmacao do user; poda de migracao no repo (42->27 entries,
100% Moodle) revelou shadowing do importer. Baseline eval: 14/25 = 56.0%.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JaucN6kPaQ8HC255wveGuh
</commit_message>
<xml_diff>
--- a/docs/reports/gold_templates/gold_TCC_rotular.xlsx
+++ b/docs/reports/gold_templates/gold_TCC_rotular.xlsx
@@ -2,16 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rotulagem" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gabarito dos Blocos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -27,7 +26,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -39,12 +40,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
+        <fgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -80,7 +81,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -444,7 +445,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G43"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>
@@ -511,9 +512,17 @@
           <t>3D Matching</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr"/>
-      <c r="F2" s="5" t="inlineStr"/>
-      <c r="G2" s="6" t="inlineStr"/>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>bloco-24</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -534,11 +543,19 @@
           <t>3DM Caetano, Gabriel e Gustavo</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-    </row>
-    <row r="4">
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>bloco-24</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="n"/>
+    </row>
+    <row r="4" ht="28.8" customHeight="1">
       <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
@@ -557,11 +574,23 @@
           <t>Aula 01 Apresentação da Disciplina, Revisão de Teoria de Conjuntos e Enumerabilidade</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-    </row>
-    <row r="5">
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>bloco-01</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>fix off-by-one 2026-07-01 (user-confirmado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28.8" customHeight="1">
       <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
@@ -580,11 +609,19 @@
           <t>Aula 02 Conjuntos Enumeráveis e Não Enumeráveis; Argumento da Diagonalização de Cantor</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-    </row>
-    <row r="6">
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>bloco-02</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="28.8" customHeight="1">
       <c r="A6" s="3" t="n">
         <v>5</v>
       </c>
@@ -603,11 +640,19 @@
           <t>Aula 03 Funções Recursivas Primitivas e Composição de Funções</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-    </row>
-    <row r="7">
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>bloco-03</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="28.8" customHeight="1">
       <c r="A7" s="3" t="n">
         <v>6</v>
       </c>
@@ -626,11 +671,19 @@
           <t>Aula 04 Funções Computáveis Funções Recursivas Parciais</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-    </row>
-    <row r="8">
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>bloco-03</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="28.8" customHeight="1">
       <c r="A8" s="3" t="n">
         <v>7</v>
       </c>
@@ -649,9 +702,17 @@
           <t>Aula 04 Funções Computáveis Funções Recursivas Parciais</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr"/>
-      <c r="F8" s="5" t="inlineStr"/>
-      <c r="G8" s="6" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>bloco-03</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -672,11 +733,23 @@
           <t>Aula 05 Minimização de Funções Recursivas Parciais</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr"/>
-      <c r="F9" s="5" t="inlineStr"/>
-      <c r="G9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10">
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>bloco-03</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>fix off-by-one 2026-07-01 (user-confirmado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="43.2" customHeight="1">
       <c r="A10" s="3" t="n">
         <v>9</v>
       </c>
@@ -695,11 +768,23 @@
           <t>Aula 06 Revisão Alfabeto, Cadeia, Linguagem, Hierarquia de Chomsky, Lemas e Propriedades de Autômatos</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr"/>
-      <c r="F10" s="5" t="inlineStr"/>
-      <c r="G10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11">
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>bloco-05</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>fix off-by-one 2026-07-01 (user-confirmado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="43.2" customHeight="1">
       <c r="A11" s="3" t="n">
         <v>10</v>
       </c>
@@ -718,11 +803,23 @@
           <t>Aula 06 Revisão Alfabeto, Cadeia, Linguagem, Hierarquia de Chomsky, Lemas e Propriedades de Autômatos</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr"/>
-      <c r="F11" s="5" t="inlineStr"/>
-      <c r="G11" s="6" t="inlineStr"/>
-    </row>
-    <row r="12">
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>bloco-05</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>fix off-by-one 2026-07-01 (user-confirmado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28.8" customHeight="1">
       <c r="A12" s="3" t="n">
         <v>11</v>
       </c>
@@ -741,11 +838,19 @@
           <t>Aula 07 Máquinas de Turing e Linguagens Recursivamente Enumeráveis</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr"/>
-      <c r="F12" s="5" t="inlineStr"/>
-      <c r="G12" s="6" t="inlineStr"/>
-    </row>
-    <row r="13">
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>bloco-06</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="28.8" customHeight="1">
       <c r="A13" s="3" t="n">
         <v>12</v>
       </c>
@@ -764,11 +869,23 @@
           <t>Aula 08 Máquinas de Turing como Processadoras de Funções</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr"/>
-      <c r="F13" s="5" t="inlineStr"/>
-      <c r="G13" s="6" t="inlineStr"/>
-    </row>
-    <row r="14">
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>bloco-06</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>fix off-by-one 2026-07-01 (user-confirmado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28.8" customHeight="1">
       <c r="A14" s="3" t="n">
         <v>13</v>
       </c>
@@ -787,9 +904,21 @@
           <t>Aula 08 Maquinas de Turing como Processadores de Funções</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr"/>
-      <c r="F14" s="5" t="inlineStr"/>
-      <c r="G14" s="6" t="inlineStr"/>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>bloco-06</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>fix off-by-one 2026-07-01 (user-confirmado)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
@@ -810,11 +939,19 @@
           <t>Aula 09 Variações de Máquinas de Turing</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr"/>
-      <c r="F15" s="5" t="inlineStr"/>
-      <c r="G15" s="6" t="inlineStr"/>
-    </row>
-    <row r="16">
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>bloco-08</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="n"/>
+    </row>
+    <row r="16" ht="28.8" customHeight="1">
       <c r="A16" s="3" t="n">
         <v>15</v>
       </c>
@@ -833,11 +970,19 @@
           <t>Aula 10 Linguagens Reconhecı́veis e Linguagens Decidı́veis</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr"/>
-      <c r="F16" s="5" t="inlineStr"/>
-      <c r="G16" s="6" t="inlineStr"/>
-    </row>
-    <row r="17">
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>bloco-09</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="n"/>
+    </row>
+    <row r="17" ht="28.8" customHeight="1">
       <c r="A17" s="3" t="n">
         <v>16</v>
       </c>
@@ -856,11 +1001,19 @@
           <t>Aula 10 Linguagens Reconhecı́veis e Linguagens Decidı́veis</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr"/>
-      <c r="F17" s="5" t="inlineStr"/>
-      <c r="G17" s="6" t="inlineStr"/>
-    </row>
-    <row r="18">
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>bloco-09</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="n"/>
+    </row>
+    <row r="18" ht="28.8" customHeight="1">
       <c r="A18" s="3" t="n">
         <v>17</v>
       </c>
@@ -879,11 +1032,19 @@
           <t>Aula 11 O Problema da Parada (Halting Problem, Halteproblem)</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr"/>
-      <c r="F18" s="5" t="inlineStr"/>
-      <c r="G18" s="6" t="inlineStr"/>
-    </row>
-    <row r="19">
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>bloco-10</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="n"/>
+    </row>
+    <row r="19" ht="28.8" customHeight="1">
       <c r="A19" s="3" t="n">
         <v>18</v>
       </c>
@@ -902,9 +1063,17 @@
           <t>Aula 11 O Problema da Parada (Halting Problem, Halteproblem)</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr"/>
-      <c r="F19" s="5" t="inlineStr"/>
-      <c r="G19" s="6" t="inlineStr"/>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>bloco-10</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -925,9 +1094,17 @@
           <t>Aula 12 Entscheidungsproblem</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr"/>
-      <c r="F20" s="5" t="inlineStr"/>
-      <c r="G20" s="6" t="inlineStr"/>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>bloco-11</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -948,9 +1125,17 @@
           <t>Aula 12 Entscheidungsproblem</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr"/>
-      <c r="F21" s="5" t="inlineStr"/>
-      <c r="G21" s="6" t="inlineStr"/>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>bloco-11</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -971,9 +1156,17 @@
           <t>Aula 13 Teorema de Rice</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr"/>
-      <c r="F22" s="5" t="inlineStr"/>
-      <c r="G22" s="6" t="inlineStr"/>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>bloco-12</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -994,9 +1187,17 @@
           <t>Aula 13 Teorema de Rice</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr"/>
-      <c r="F23" s="5" t="inlineStr"/>
-      <c r="G23" s="6" t="inlineStr"/>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>bloco-12</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -1017,9 +1218,17 @@
           <t>Aula 14 Problema da Correspondência de Post</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr"/>
-      <c r="F24" s="5" t="inlineStr"/>
-      <c r="G24" s="6" t="inlineStr"/>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>bloco-13</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -1040,9 +1249,17 @@
           <t>Aula 15 Teoremas de Incompletude de Gödel</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr"/>
-      <c r="F25" s="5" t="inlineStr"/>
-      <c r="G25" s="6" t="inlineStr"/>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>bloco-14</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -1063,9 +1280,17 @@
           <t>Aula 16 Classes de Problemas e Complexidade</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr"/>
-      <c r="F26" s="5" t="inlineStr"/>
-      <c r="G26" s="6" t="inlineStr"/>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>bloco-19</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
@@ -1086,9 +1311,17 @@
           <t>Aula 16 Classes de Problemas e Complexidade</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr"/>
-      <c r="F27" s="5" t="inlineStr"/>
-      <c r="G27" s="6" t="inlineStr"/>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>bloco-19</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -1109,9 +1342,17 @@
           <t>Aula 16 Exemplo de Prova para Revisão</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr"/>
-      <c r="F28" s="5" t="inlineStr"/>
-      <c r="G28" s="6" t="inlineStr"/>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>bloco-16</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -1132,9 +1373,17 @@
           <t>Aula 17 Complexidade de Tempo Classes P e NP</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr"/>
-      <c r="F29" s="5" t="inlineStr"/>
-      <c r="G29" s="6" t="inlineStr"/>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>bloco-19</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -1155,9 +1404,17 @@
           <t>Aula 17 NP Completude</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr"/>
-      <c r="F30" s="5" t="inlineStr"/>
-      <c r="G30" s="6" t="inlineStr"/>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>bloco-22</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -1178,11 +1435,19 @@
           <t>Aula 17 NP Completude</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr"/>
-      <c r="F31" s="5" t="inlineStr"/>
-      <c r="G31" s="6" t="inlineStr"/>
-    </row>
-    <row r="32">
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>bloco-22</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="n"/>
+    </row>
+    <row r="32" ht="28.8" customHeight="1">
       <c r="A32" s="3" t="n">
         <v>31</v>
       </c>
@@ -1201,9 +1466,17 @@
           <t>Aula07 Máquinas de Turing e Linguagens Recursivamente Enumeráveis</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr"/>
-      <c r="F32" s="5" t="inlineStr"/>
-      <c r="G32" s="6" t="inlineStr"/>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>bloco-06</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
@@ -1224,9 +1497,17 @@
           <t>Cubic 3 Edge Coloring</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr"/>
-      <c r="F33" s="5" t="inlineStr"/>
-      <c r="G33" s="6" t="inlineStr"/>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>bloco-24</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
@@ -1247,9 +1528,17 @@
           <t>Enunciado T1</t>
         </is>
       </c>
-      <c r="E34" s="5" t="inlineStr"/>
-      <c r="F34" s="5" t="inlineStr"/>
-      <c r="G34" s="6" t="inlineStr"/>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>bloco-04</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
@@ -1270,9 +1559,17 @@
           <t>Enunciado T2</t>
         </is>
       </c>
-      <c r="E35" s="5" t="inlineStr"/>
-      <c r="F35" s="5" t="inlineStr"/>
-      <c r="G35" s="6" t="inlineStr"/>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>bloco-23</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -1293,9 +1590,17 @@
           <t>Integer Programming 00</t>
         </is>
       </c>
-      <c r="E36" s="5" t="inlineStr"/>
-      <c r="F36" s="5" t="inlineStr"/>
-      <c r="G36" s="6" t="inlineStr"/>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>bloco-24</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
@@ -1316,9 +1621,17 @@
           <t>Plano de Ensino</t>
         </is>
       </c>
-      <c r="E37" s="5" t="inlineStr"/>
-      <c r="F37" s="5" t="inlineStr"/>
-      <c r="G37" s="6" t="inlineStr"/>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>bloco-01</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
@@ -1339,9 +1652,17 @@
           <t>Problema Weighted Max Cut</t>
         </is>
       </c>
-      <c r="E38" s="5" t="inlineStr"/>
-      <c r="F38" s="5" t="inlineStr"/>
-      <c r="G38" s="6" t="inlineStr"/>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>bloco-24</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
@@ -1362,11 +1683,19 @@
           <t>Programação Inteira 01 20260617 154423 0000</t>
         </is>
       </c>
-      <c r="E39" s="5" t="inlineStr"/>
-      <c r="F39" s="5" t="inlineStr"/>
-      <c r="G39" s="6" t="inlineStr"/>
-    </row>
-    <row r="40">
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>bloco-24</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="n"/>
+    </row>
+    <row r="40" ht="28.8" customHeight="1">
       <c r="A40" s="3" t="n">
         <v>39</v>
       </c>
@@ -1385,11 +1714,19 @@
           <t>Referência REDUCIBILITY AMONG COMBINATORIAL PROBLEMS</t>
         </is>
       </c>
-      <c r="E40" s="5" t="inlineStr"/>
-      <c r="F40" s="5" t="inlineStr"/>
-      <c r="G40" s="6" t="inlineStr"/>
-    </row>
-    <row r="41">
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>bloco-23</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="n"/>
+    </row>
+    <row r="41" ht="28.8" customHeight="1">
       <c r="A41" s="3" t="n">
         <v>40</v>
       </c>
@@ -1408,9 +1745,21 @@
           <t>Revisão Alfabeto, Cadeia, Linguagem, Hierarquia de Chomsky, Lemas e Propriedades de Autômatos</t>
         </is>
       </c>
-      <c r="E41" s="5" t="inlineStr"/>
-      <c r="F41" s="5" t="inlineStr"/>
-      <c r="G41" s="6" t="inlineStr"/>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>bloco-05</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>fix off-by-one 2026-07-01 (user-confirmado)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
@@ -1431,9 +1780,17 @@
           <t>T1 Enunciado</t>
         </is>
       </c>
-      <c r="E42" s="5" t="inlineStr"/>
-      <c r="F42" s="5" t="inlineStr"/>
-      <c r="G42" s="6" t="inlineStr"/>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>bloco-04</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n">
@@ -1454,16 +1811,20 @@
           <t>Trabalho T2 Enunciado</t>
         </is>
       </c>
-      <c r="E43" s="5" t="inlineStr"/>
-      <c r="F43" s="5" t="inlineStr"/>
-      <c r="G43" s="6" t="inlineStr"/>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>bloco-23</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0"/>
-  <dataValidations count="2">
-    <dataValidation sqref="E2:E43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Escolha um subtópico da lista (ou N/A / não sei)." prompt="Selecione o subtópico correto (SARC)." type="list">
-      <formula1>'Gabarito dos Blocos'!$F$2:$F$34</formula1>
-    </dataValidation>
+  <dataValidations count="1">
     <dataValidation sqref="F2:F43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" prompt="Sua confiança na resposta." type="list">
       <formula1>"alta,média,baixa"</formula1>
     </dataValidation>
@@ -1479,7 +1840,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F34"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -1509,7 +1870,6 @@
           <t>tipo</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr"/>
       <c r="F1" t="inlineStr">
         <is>
           <t>_opcoes</t>
@@ -1570,7 +1930,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="28.8" customHeight="1">
       <c r="A4" t="inlineStr">
         <is>
           <t>bloco-03</t>
@@ -1624,7 +1984,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="28.8" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
           <t>bloco-05</t>
@@ -1651,7 +2011,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="28.8" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
           <t>bloco-06</t>
@@ -2002,7 +2362,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="28.8" customHeight="1">
       <c r="A20" t="inlineStr">
         <is>
           <t>bloco-19</t>
@@ -2083,7 +2443,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="28.8" customHeight="1">
       <c r="A23" t="inlineStr">
         <is>
           <t>bloco-22</t>
@@ -2137,7 +2497,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="28.8" customHeight="1">
       <c r="A25" t="inlineStr">
         <is>
           <t>bloco-24</t>

</xml_diff>